<commit_message>
modified Functional TS to make it relevanct for currect testing
</commit_message>
<xml_diff>
--- a/docs/Functional_TestSuite.xlsx
+++ b/docs/Functional_TestSuite.xlsx
@@ -9,22 +9,21 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="75" windowWidth="18195" windowHeight="11820" activeTab="2"/>
+    <workbookView xWindow="480" yWindow="75" windowWidth="18195" windowHeight="11820" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Test Suite Overview" sheetId="1" r:id="rId1"/>
+    <sheet name="Test Execution Summary" sheetId="6" r:id="rId9"/>
+    <sheet name="Defect Log" sheetId="5" r:id="rId8"/>
     <sheet name="Test Data" sheetId="4" r:id="rId7"/>
-    <sheet name="Defect Log" sheetId="5" r:id="rId8"/>
-    <sheet name="Test Execution Summary" sheetId="6" r:id="rId9"/>
-    <sheet name="Login" sheetId="2" r:id="rId2"/>
+    <sheet name="Authentication" sheetId="2" r:id="rId2"/>
+    <sheet name="Logout" sheetId="16" r:id="rId18"/>
     <sheet name="User Management" sheetId="14" r:id="rId10"/>
+    <sheet name="Leave" sheetId="15" r:id="rId3"/>
     <sheet name="PIM" sheetId="7" r:id="rId11"/>
-    <sheet name="Leave" sheetId="15" r:id="rId3"/>
     <sheet name="Time" sheetId="10" r:id="rId13"/>
     <sheet name="Performance" sheetId="11" r:id="rId14"/>
     <sheet name="Dashboard" sheetId="12" r:id="rId15"/>
-    <sheet name="Logout" sheetId="16" r:id="rId18"/>
-    <sheet name="Recruitment" sheetId="9" r:id="rId17"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -737,12 +736,188 @@
 4. Enter the existing username
 5. Click 'Reset Password' button</t>
   </si>
+  <si>
+    <t>504 Gateway Time-out occurs after clicking 'Reset Password' on OrangeHRM login</t>
+  </si>
+  <si>
+    <t>When a user attempts to reset their password using the 'Forgot Password' functionality, the system returns a 504 Gateway Time-out error.</t>
+  </si>
+  <si>
+    <t>Password reset request should complete successfully.
+User should see confirmation message - 'Reset Password link sent successfully'
+No server error (504) should occur.</t>
+  </si>
+  <si>
+    <t>1. Navigate to Leave Tab
+2. Click on 'Approve' button</t>
+  </si>
+  <si>
+    <t>Employee can login with valid credentials</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>New Admin</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Not Started</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>P0</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>IamEmployeeJohn</t>
+  </si>
+  <si>
+    <t>IAmEmployee123</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Authentication</t>
+  </si>
+  <si>
+    <t>Valid users (Admin/ESS) can log in with correct credentials</t>
+  </si>
+  <si>
+    <t>Login with valid Admin credentials should redirect to Admin Dashboard</t>
+  </si>
+  <si>
+    <t>User is authenticated successfully.
+User is redirected to the Dashboard page.</t>
+  </si>
+  <si>
+    <t>Error message should be displayed when an invalid password is entered</t>
+  </si>
+  <si>
+    <t>Authentication is rejected.
+User remains on the Login page.
+Error message "Invalid credentials" is displayed.</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-3</t>
+  </si>
+  <si>
+    <t>Error message should be displayed when an invalid username is entered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to the Login page. 
+2. Enter an invalid username. 
+3. Enter a valid password. 
+4. Click the 'Login' button.  </t>
+  </si>
+  <si>
+    <t>Username: User
+Password: WrongPass</t>
+  </si>
+  <si>
+    <t>Username: User
+Password: admin123</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-4</t>
+  </si>
+  <si>
+    <t>Hint message should be displayed when trying to login with an empty username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to the Login page. 
+2. Leave username field empty.. 
+3. Enter a valid password. 
+4. Click the 'Login' button.  </t>
+  </si>
+  <si>
+    <t>Username: User
+Password: admin124</t>
+  </si>
+  <si>
+    <t>Username: Password: admin124</t>
+  </si>
+  <si>
+    <t>Username: 
+Password: admin124</t>
+  </si>
+  <si>
+    <t>Authentication is rejected.
+User remains on the Login page.
+int message *"Required"* is displayed next to Username field..</t>
+  </si>
+  <si>
+    <t>Authentication is rejected.
+User remains on the Login page.
+Hint message "Required" is displayed next to Username field..</t>
+  </si>
+  <si>
+    <t>Hint message should be displayed when trying to login with an empty password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Username: Admin
+Password: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to the Login page. 
+2. Enter a valid username. 
+3. Enter a valid password. 
+4. Click the 'Login' button.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to the Login page. 
+2. Leave username field empty..
+3. Enter a valid password. 
+4. Click the 'Login' button.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to the Login page. 
+2. Enter a valid username. 
+3. Leave password field empty.
+4. Click the 'Login' button.  </t>
+  </si>
+  <si>
+    <t>Authentication is rejected.
+User remains on the Login page.
+Hint message "Required" is displayed next to Password field.</t>
+  </si>
+  <si>
+    <t>Authentication is rejected.
+User remains on the Login page.
+Hint message "Required" is displayed next to Username field.</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-006</t>
+  </si>
+  <si>
+    <t>Logged-in user can successfully log out and the session is terminated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click the user profile icon in the top-right corner. 
+2. Select 'Logout' from the dropdown menu. </t>
+  </si>
+  <si>
+    <t>1. User is successfully logged out.
+2. User is redirected to the Login page.
+3. Application session is terminated.
+4. Protected pages are no longer accessible without authentication.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -754,6 +929,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <color rgb="FFFF0000"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -843,7 +1026,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="2" applyFill="1" xfId="0"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="3" applyFill="1" xfId="0"/>
@@ -865,6 +1048,7 @@
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="12" applyFill="1" xfId="0"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="13" applyFill="1" xfId="0"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="14" applyFill="1" xfId="0"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="2" applyFont="1" fillId="0" applyFill="1" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1204,7 +1388,13 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>221</v>
+      </c>
+      <c r="C2" t="s">
+        <v>212</v>
+      </c>
+      <c r="D2" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="3">
@@ -1214,6 +1404,12 @@
       <c r="B3" t="s">
         <v>40</v>
       </c>
+      <c r="C3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D3" t="s">
+        <v>215</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
@@ -1222,6 +1418,12 @@
       <c r="B4" t="s">
         <v>41</v>
       </c>
+      <c r="C4" t="s">
+        <v>213</v>
+      </c>
+      <c r="D4" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
@@ -1230,6 +1432,12 @@
       <c r="B5" t="s">
         <v>42</v>
       </c>
+      <c r="C5" t="s">
+        <v>212</v>
+      </c>
+      <c r="D5" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -1238,6 +1446,12 @@
       <c r="B6" t="s">
         <v>43</v>
       </c>
+      <c r="C6" t="s">
+        <v>213</v>
+      </c>
+      <c r="D6" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
@@ -1246,6 +1460,12 @@
       <c r="B7" t="s">
         <v>44</v>
       </c>
+      <c r="C7" t="s">
+        <v>213</v>
+      </c>
+      <c r="D7" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
@@ -1254,6 +1474,12 @@
       <c r="B8" t="s">
         <v>45</v>
       </c>
+      <c r="C8" t="s">
+        <v>213</v>
+      </c>
+      <c r="D8" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
@@ -1261,6 +1487,12 @@
       </c>
       <c r="B9" t="s">
         <v>46</v>
+      </c>
+      <c r="C9" t="s">
+        <v>214</v>
+      </c>
+      <c r="D9" t="s">
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -1292,14 +1524,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
@@ -1348,13 +1572,10 @@
         <v>4</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L1" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="2" ht="28.5">
+    <row r="2" ht="123">
       <c r="A2" t="s">
         <v>129</v>
       </c>
@@ -1362,26 +1583,25 @@
         <v>47</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>130</v>
+        <v>248</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>131</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="F2" s="10"/>
+        <v>249</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>63</v>
+      </c>
       <c r="G2" s="10" t="s">
-        <v>133</v>
+        <v>250</v>
       </c>
       <c r="I2" s="7" t="s">
         <v>105</v>
       </c>
       <c r="J2" t="s">
-        <v>134</v>
-      </c>
-      <c r="K2" t="s">
-        <v>135</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3">
@@ -1450,9 +1670,6 @@
         <v>4</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L1" s="2" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1464,7 +1681,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>146</v>
+        <v>223</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>59</v>
@@ -1476,7 +1693,7 @@
         <v>63</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>64</v>
+        <v>224</v>
       </c>
       <c r="I2" s="7" t="s">
         <v>105</v>
@@ -1484,11 +1701,8 @@
       <c r="J2" t="s">
         <v>67</v>
       </c>
-      <c r="K2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" ht="123">
+    </row>
+    <row r="3" ht="136.5">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -1496,31 +1710,28 @@
         <v>8</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>95</v>
+        <v>225</v>
+      </c>
+      <c r="D3" t="s">
+        <v>80</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>94</v>
+        <v>226</v>
       </c>
       <c r="I3" s="7" t="s">
         <v>105</v>
       </c>
       <c r="J3" t="s">
-        <v>67</v>
-      </c>
-      <c r="K3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="4" ht="136.5">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" ht="109.5">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -1528,31 +1739,26 @@
         <v>8</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>148</v>
+        <v>228</v>
       </c>
       <c r="D4" t="s">
         <v>80</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>81</v>
+        <v>229</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>82</v>
+        <v>231</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>105</v>
-      </c>
+        <v>226</v>
+      </c>
+      <c r="I4" s="7"/>
       <c r="J4" t="s">
         <v>84</v>
       </c>
-      <c r="K4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" ht="123">
+    </row>
+    <row r="5" ht="109.5">
       <c r="A5" t="s">
         <v>160</v>
       </c>
@@ -1560,31 +1766,26 @@
         <v>8</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>138</v>
+        <v>233</v>
+      </c>
+      <c r="D5" t="s">
+        <v>80</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>62</v>
+        <v>243</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>141</v>
+        <v>237</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>105</v>
-      </c>
+        <v>246</v>
+      </c>
+      <c r="I5" s="7"/>
       <c r="J5" t="s">
-        <v>67</v>
-      </c>
-      <c r="K5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" ht="177">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" ht="109.5">
       <c r="A6" t="s">
         <v>161</v>
       </c>
@@ -1592,32 +1793,61 @@
         <v>8</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>172</v>
+        <v>240</v>
       </c>
       <c r="D6" t="s">
         <v>80</v>
       </c>
       <c r="E6" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="I6" s="7"/>
+      <c r="J6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" ht="177">
+      <c r="A7" t="s">
+        <v>247</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="D7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F7" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G7" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H7" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="I7" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="J6" t="s">
-        <v>67</v>
-      </c>
-      <c r="K6" t="s">
-        <v>67</v>
-      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1672,9 +1902,6 @@
         <v>4</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L1" s="2" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1706,9 +1933,6 @@
       <c r="J2" t="s">
         <v>84</v>
       </c>
-      <c r="K2" t="s">
-        <v>85</v>
-      </c>
     </row>
     <row r="3" ht="55.5">
       <c r="A3" t="s">
@@ -1724,7 +1948,7 @@
         <v>123</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>124</v>
+        <v>208</v>
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="10" t="s">
@@ -1735,9 +1959,6 @@
       </c>
       <c r="J3" t="s">
         <v>84</v>
-      </c>
-      <c r="K3" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="4">
@@ -1755,9 +1976,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="14.2578125" customWidth="1"/>
-    <col min="2" max="2" width="10.22265625" customWidth="1"/>
-    <col min="3" max="3" width="11.43359375" customWidth="1"/>
+    <col min="1" max="1" width="24.48046875" customWidth="1"/>
+    <col min="2" max="2" width="26.5" customWidth="1"/>
+    <col min="3" max="3" width="18.29296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1780,6 +2001,17 @@
       </c>
       <c r="C2" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C3" t="s">
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -1851,7 +2083,7 @@
         <v>171</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>186</v>
+        <v>205</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -1866,7 +2098,7 @@
         <v>203</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>204</v>
@@ -1875,13 +2107,13 @@
         <v>196</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="K2" s="10" t="s">
         <v>200</v>
       </c>
       <c r="L2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M2" t="s">
         <v>67</v>
@@ -1895,6 +2127,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="16.0078125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
@@ -1914,6 +2149,186 @@
       </c>
       <c r="F1" s="12" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B2">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>5</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="s">
+        <v>220</v>
+      </c>
+      <c r="B10" s="17">
+        <v>12</v>
+      </c>
+      <c r="C10" s="17">
+        <v>10</v>
+      </c>
+      <c r="D10" s="17">
+        <v>1</v>
+      </c>
+      <c r="E10" s="17">
+        <v>0</v>
+      </c>
+      <c r="F10" s="17">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1969,9 +2384,6 @@
         <v>4</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L1" s="2" t="s">
         <v>55</v>
       </c>
     </row>
@@ -2003,9 +2415,6 @@
       <c r="J2" t="s">
         <v>67</v>
       </c>
-      <c r="K2" t="s">
-        <v>85</v>
-      </c>
     </row>
     <row r="3" ht="55.5">
       <c r="A3" t="s">
@@ -2035,9 +2444,6 @@
       <c r="J3" t="s">
         <v>67</v>
       </c>
-      <c r="K3" t="s">
-        <v>68</v>
-      </c>
     </row>
     <row r="4" ht="150">
       <c r="A4" t="s">
@@ -2066,9 +2472,6 @@
       </c>
       <c r="J4" t="s">
         <v>67</v>
-      </c>
-      <c r="K4" t="s">
-        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>